<commit_message>
auto: 2026-04-01 18:05 (2 files)
</commit_message>
<xml_diff>
--- a/тексти/хейхо/HeyHo Emails Summary.xlsx
+++ b/тексти/хейхо/HeyHo Emails Summary.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Oink Oink Oink at HeyHo</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Oink Oink Oink at HeyHo</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Oink Oink Oink at HeyHo</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Le Bandit at HeyHo</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Oink Oink Oink at HeyHo</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Le Bandit at HeyHo</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Le Bandit at HeyHo</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Le Bandit at HeyHo</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Le Bandit at HeyHo</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Oink Oink Oink Ahoy</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Oink Oink Oink Ahoy</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Oink Oink Oink Ahoy</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Le Bandit Ahoy</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Oink Oink Oink Ahoy</t>
+          <t>Oink Oink Oink</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Le Bandit Ahoy</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Le Bandit Ahoy</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Le Bandit Ahoy</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Le Bandit Ahoy</t>
+          <t>Le Bandit</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>9% Cashback</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>⛈️ The storm gave back 12% Cash Back</t>
+          <t>12% Cashback</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>The deep sea brings 15% Cash Back</t>
+          <t>15% Cashback</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Hand of Midas 2 Ahoy</t>
+          <t>Hand of Midas 2</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Hand of Midas 2 Ahoy</t>
+          <t>Hand of Midas 2</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Hand of Midas 2 Ahoy</t>
+          <t>Hand of Midas 2</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Hand of Midas 2 Ahoy</t>
+          <t>Hand of Midas 2</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>45 FS</t>
+          <t>74% + 45 FS</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>55 FS</t>
+          <t>74% + 55 FS</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>55 FS</t>
+          <t>82% + 55 FS</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>55 FS</t>
+          <t>86% + 55 FS</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>65 FS</t>
+          <t>82% + 65 FS</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>65 FS</t>
+          <t>90% + 65 FS</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>80 FS</t>
+          <t>90% + 80 FS</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>90 FS</t>
+          <t>90% + 90 FS</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>20% Cash Back resets your luck</t>
+          <t>20% Cashback</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -2205,7 +2205,11 @@
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr"/>
-      <c r="D24" s="13" t="inlineStr"/>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Big Bass Splash</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -2221,7 +2225,7 @@
       <c r="C25" s="12" t="inlineStr"/>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Reactoonz 2 Ahoy</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2379,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>‍☠️ The crew got 75% from the merchant ship</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -2605,7 +2609,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>40 FS</t>
+          <t>55% + 40 FS</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -2627,7 +2631,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>40 FS</t>
+          <t>69% + 40 FS</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -2649,7 +2653,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>40 FS</t>
+          <t>77% + 40 FS</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -2671,7 +2675,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>69% + 50 FS</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -2693,7 +2697,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>77% + 50 FS</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -2715,7 +2719,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>81% + 50 FS</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -2737,7 +2741,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>60 FS</t>
+          <t>77% + 60 FS</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -2759,7 +2763,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>75 FS</t>
+          <t>85% + 75 FS</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -2781,7 +2785,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>85 FS</t>
+          <t>85% + 85 FS</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -2905,7 +2909,7 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>️ A storm of luck hit three brave sailors</t>
+          <t>A storm of luck hit three brave sailors</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr"/>
@@ -2995,7 +2999,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Sweet Bonanza Ahoy</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3039,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Gates of Olympus with a clean boost</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3051,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>150 FS</t>
+          <t>150% + 150 FS</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -3137,7 +3141,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Gates of Olympus Ahoy</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3181,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Book of Dead Ahoy</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3255,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Sweet Bonanza as a thank you</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3385,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Gates of Olympus into your account</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3407,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Gates of Olympus Ahoy</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3425,7 +3429,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>the Shining Crown</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3451,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Gates of Olympus Await You Ahoy</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3473,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Shining Crown Ahoy</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3495,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Book of Dead Ready to Launch Ahoy</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3517,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>the Sweet Bonanza</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3539,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>the Reactoonz 2</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3561,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Gates of Olympus Ahoy</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3657,7 @@
       <c r="C17" s="12" t="inlineStr"/>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Cleocatra Last Week</t>
+          <t>Cleocatra</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3749,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Gates of Olympus Ahoy</t>
+          <t>Gates of Olympus</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3771,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Book of Dead Ahoy</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3793,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Book of Dead Ahoy</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3917,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Reactoonz 2 - unleash the fun Ahoy</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3957,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Legacy of Dead - uncover secrets Ahoy</t>
+          <t>Legacy of Dead</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4037,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Shining Crown Ahoy</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4255,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Sands revealed 115% on next dep</t>
+          <t>115%</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -4269,7 +4273,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Sands revealed 120% on next dep</t>
+          <t>120%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -4323,7 +4327,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>️ A ship of silver, a captain with 120%</t>
+          <t>120%</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -4341,7 +4345,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>️ A ship of silver, a captain with 125%</t>
+          <t>125%</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -4395,7 +4399,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>️ Attack them for 130%</t>
+          <t>130%</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -4475,7 +4479,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4501,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4523,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4545,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sugar Rush 1000</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4567,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4589,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4611,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4633,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4655,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -4671,11 +4675,7 @@
           <t>ASK4MRBQY7</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>next deposit</t>
-        </is>
-      </c>
+      <c r="D12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4739,7 +4739,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -4781,11 +4781,7 @@
           <t>ASKFORMEAJ2</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>next deposit</t>
-        </is>
-      </c>
+      <c r="D17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -4805,7 +4801,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -4893,7 +4889,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -5003,7 +4999,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>next deposit</t>
+          <t>Shining Crown</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5035,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Reactoonz 2: ⭐30 Spins for a 20 € deposit Code ASKFORMORE1 ⭐50 Spins for a 30 € deposit Code ASK4MOREV7X ⭐70 Spins for 50 € or more Code ASKFORMZKQ2 The bigger the top-up</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5057,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Reactoonz 2: ⭐50 Spins for a 20 € deposit Code ASK4MOREV7X ⭐70 Spins for a 30 € deposit Code ASKFORMZKQ2 ⭐90 Spins for 50 € or more Code LEGA90 The bigger the top-up</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5079,7 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>Reactoonz 2: ⭐70 Spins for a 20 € deposit Code ASKFORMZKQ2 ⭐90 Spins for a 30 € deposit Code LEGA90 ⭐120 Spins for 50 € or more Code CROWN120 The bigger the top-up</t>
+          <t>Reactoonz 2</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5327,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>‍☠️ Third deposit: 90% at HeyHo ‍☠️</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -5349,7 +5345,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>‍☠️ Third deposit: 95% at HeyHo ‍☠️</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
@@ -5403,7 +5399,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>️ 90% on your third deposit</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -5421,7 +5417,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>️ 95% on your third deposit</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -5475,7 +5471,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Get your 95% on next deposit</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -5643,7 +5639,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Book of Dead Extra credit extends your play</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5661,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Book of Dead Extra credit extends your play</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5683,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Book of Dead Extra credit extends your play</t>
+          <t>Book of Dead</t>
         </is>
       </c>
     </row>
@@ -5733,7 +5729,7 @@
       <c r="C12" s="13" t="inlineStr"/>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Sweet Bonanza 🦈Wil*****64 – €16</t>
+          <t>Sweet Bonanza</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5947,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>☠️ 95% on Your Next Deposit Fresh from the Skull</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -6031,7 +6027,7 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6049,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6075,7 +6071,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6093,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6115,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6137,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6159,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6181,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6193,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>70% + 50 FS</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -6207,7 +6203,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6215,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>90% + 50 FS</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -6229,7 +6225,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6237,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>50 FS</t>
+          <t>100% + 50 FS</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -6251,7 +6247,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6259,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>60 FS</t>
+          <t>90% + 60 FS</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -6273,7 +6269,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6281,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>60 FS</t>
+          <t>100% + 60 FS</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -6295,7 +6291,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6303,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>60 FS</t>
+          <t>105% + 60 FS</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -6317,7 +6313,7 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6325,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>70 FS</t>
+          <t>100% + 70 FS</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -6339,7 +6335,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6347,7 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>70 FS</t>
+          <t>110% + 70 FS</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -6361,7 +6357,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6373,7 +6369,7 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>90 FS</t>
+          <t>110% + 90 FS</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
@@ -6383,7 +6379,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>this wild</t>
+          <t>Wolf Gold</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6419,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6441,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6467,7 +6463,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6485,7 @@
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6507,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Starburst Ahoy</t>
+          <t>Starburst</t>
         </is>
       </c>
     </row>
@@ -6533,7 +6529,7 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6555,7 +6551,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6573,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Big Bass Splash Ahoy</t>
+          <t>Big Bass Splash</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 2026-04-01 18:06 (2 files)
</commit_message>
<xml_diff>
--- a/тексти/хейхо/HeyHo Emails Summary.xlsx
+++ b/тексти/хейхо/HeyHo Emails Summary.xlsx
@@ -5113,11 +5113,7 @@
           <t>ASKFORMORE1</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>Your Second Deposit Ahoy</t>
-        </is>
-      </c>
+      <c r="D33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -5135,11 +5131,7 @@
           <t>ASK4MOREV7X</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>Your Second Deposit Ahoy</t>
-        </is>
-      </c>
+      <c r="D34" s="13" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
@@ -5157,11 +5149,7 @@
           <t>ASKFORMZKQ2</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>Your Second Deposit Ahoy</t>
-        </is>
-      </c>
+      <c r="D35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="13" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-04-01 19:22 (2 files)
</commit_message>
<xml_diff>
--- a/тексти/хейхо/HeyHo Emails Summary.xlsx
+++ b/тексти/хейхо/HeyHo Emails Summary.xlsx
@@ -1884,7 +1884,11 @@
           <t>COIN457</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -1902,7 +1906,11 @@
           <t>COIN557</t>
         </is>
       </c>
-      <c r="D8" s="11" t="n"/>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1920,7 +1928,11 @@
           <t>COIN558</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n"/>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -1938,7 +1950,11 @@
           <t>COIN556</t>
         </is>
       </c>
-      <c r="D10" s="11" t="n"/>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1956,7 +1972,11 @@
           <t>COIN658</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n"/>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -1974,7 +1994,11 @@
           <t>COIN659</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1992,7 +2016,11 @@
           <t>COIN809</t>
         </is>
       </c>
-      <c r="D13" s="10" t="n"/>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -2010,7 +2038,11 @@
           <t>CAND909</t>
         </is>
       </c>
-      <c r="D14" s="11" t="n"/>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>3 Coins</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -4680,7 +4712,11 @@
           <t>ASK4MRBQY7</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>27 Dice</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -4786,7 +4822,11 @@
           <t>ASKFORMEAJ2</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n"/>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>20 Power Hot Dice</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">

</xml_diff>